<commit_message>
Gameweek 9 Results Commit
</commit_message>
<xml_diff>
--- a/Predictions 2(Records).xlsx
+++ b/Predictions 2(Records).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git-Folder\Premier-League-Predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F906175-95C4-4F47-91F9-FCFFF87F568E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FACF32F3-9BBB-4C84-8EF9-6C5B62D3904E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" xr2:uid="{B97D2B54-78E2-448B-A9CF-77B7E3BC2EA1}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="68">
   <si>
     <t>Goals</t>
   </si>
@@ -204,6 +204,39 @@
   </si>
   <si>
     <t>EVE vs TOT</t>
+  </si>
+  <si>
+    <t>Match Week 10</t>
+  </si>
+  <si>
+    <t>BHA vs LEE</t>
+  </si>
+  <si>
+    <t>CRY vs BRE</t>
+  </si>
+  <si>
+    <t>FUL vs WOL</t>
+  </si>
+  <si>
+    <t>BUR vs ARS</t>
+  </si>
+  <si>
+    <t>NOF vs MUN</t>
+  </si>
+  <si>
+    <t>TOT vs CHE</t>
+  </si>
+  <si>
+    <t>LIV vs AVL</t>
+  </si>
+  <si>
+    <t>WHU vs NCU</t>
+  </si>
+  <si>
+    <t>MCI vs BOU</t>
+  </si>
+  <si>
+    <t>SUN vs EVE</t>
   </si>
 </sst>
 </file>
@@ -831,10 +864,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1212,34 +1245,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA341253-1EAB-4104-BE4B-374BC158237A}">
-  <dimension ref="A1:W68"/>
+  <dimension ref="A1:W85"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:23" ht="24" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13"/>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13"/>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13"/>
-      <c r="T1" s="13"/>
-      <c r="U1" s="13"/>
-      <c r="V1" s="13"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
+      <c r="T1" s="12"/>
+      <c r="U1" s="12"/>
+      <c r="V1" s="12"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
@@ -1639,37 +1672,37 @@
       </c>
     </row>
     <row r="17" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="U17" s="12" t="s">
+      <c r="U17" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="V17" s="12"/>
+      <c r="V17" s="13"/>
       <c r="W17" s="11">
         <f>W16</f>
         <v>-0.74000000000000021</v>
       </c>
     </row>
     <row r="18" spans="1:23" ht="24" x14ac:dyDescent="0.4">
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
-      <c r="K18" s="13"/>
-      <c r="L18" s="13"/>
-      <c r="M18" s="13"/>
-      <c r="N18" s="13"/>
-      <c r="O18" s="13"/>
-      <c r="P18" s="13"/>
-      <c r="Q18" s="13"/>
-      <c r="R18" s="13"/>
-      <c r="S18" s="13"/>
-      <c r="T18" s="13"/>
-      <c r="U18" s="13"/>
-      <c r="V18" s="13"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="12"/>
+      <c r="P18" s="12"/>
+      <c r="Q18" s="12"/>
+      <c r="R18" s="12"/>
+      <c r="S18" s="12"/>
+      <c r="T18" s="12"/>
+      <c r="U18" s="12"/>
+      <c r="V18" s="12"/>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
@@ -2109,37 +2142,37 @@
       </c>
     </row>
     <row r="34" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="U34" s="12" t="s">
+      <c r="U34" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="V34" s="12"/>
+      <c r="V34" s="13"/>
       <c r="W34" s="11">
         <f>W33+W17</f>
         <v>-0.58000000000000007</v>
       </c>
     </row>
     <row r="35" spans="1:23" ht="24" x14ac:dyDescent="0.4">
-      <c r="D35" s="13" t="s">
+      <c r="D35" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="13"/>
-      <c r="J35" s="13"/>
-      <c r="K35" s="13"/>
-      <c r="L35" s="13"/>
-      <c r="M35" s="13"/>
-      <c r="N35" s="13"/>
-      <c r="O35" s="13"/>
-      <c r="P35" s="13"/>
-      <c r="Q35" s="13"/>
-      <c r="R35" s="13"/>
-      <c r="S35" s="13"/>
-      <c r="T35" s="13"/>
-      <c r="U35" s="13"/>
-      <c r="V35" s="13"/>
+      <c r="E35" s="12"/>
+      <c r="F35" s="12"/>
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="12"/>
+      <c r="K35" s="12"/>
+      <c r="L35" s="12"/>
+      <c r="M35" s="12"/>
+      <c r="N35" s="12"/>
+      <c r="O35" s="12"/>
+      <c r="P35" s="12"/>
+      <c r="Q35" s="12"/>
+      <c r="R35" s="12"/>
+      <c r="S35" s="12"/>
+      <c r="T35" s="12"/>
+      <c r="U35" s="12"/>
+      <c r="V35" s="12"/>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.25">
       <c r="D36" t="s">
@@ -2665,37 +2698,37 @@
       </c>
     </row>
     <row r="51" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="U51" s="12" t="s">
+      <c r="U51" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="V51" s="12"/>
+      <c r="V51" s="13"/>
       <c r="W51" s="11">
         <f>W34+W50</f>
         <v>0.82000000000000028</v>
       </c>
     </row>
     <row r="52" spans="1:23" ht="24" x14ac:dyDescent="0.4">
-      <c r="D52" s="13" t="s">
+      <c r="D52" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="E52" s="13"/>
-      <c r="F52" s="13"/>
-      <c r="G52" s="13"/>
-      <c r="H52" s="13"/>
-      <c r="I52" s="13"/>
-      <c r="J52" s="13"/>
-      <c r="K52" s="13"/>
-      <c r="L52" s="13"/>
-      <c r="M52" s="13"/>
-      <c r="N52" s="13"/>
-      <c r="O52" s="13"/>
-      <c r="P52" s="13"/>
-      <c r="Q52" s="13"/>
-      <c r="R52" s="13"/>
-      <c r="S52" s="13"/>
-      <c r="T52" s="13"/>
-      <c r="U52" s="13"/>
-      <c r="V52" s="13"/>
+      <c r="E52" s="12"/>
+      <c r="F52" s="12"/>
+      <c r="G52" s="12"/>
+      <c r="H52" s="12"/>
+      <c r="I52" s="12"/>
+      <c r="J52" s="12"/>
+      <c r="K52" s="12"/>
+      <c r="L52" s="12"/>
+      <c r="M52" s="12"/>
+      <c r="N52" s="12"/>
+      <c r="O52" s="12"/>
+      <c r="P52" s="12"/>
+      <c r="Q52" s="12"/>
+      <c r="R52" s="12"/>
+      <c r="S52" s="12"/>
+      <c r="T52" s="12"/>
+      <c r="U52" s="12"/>
+      <c r="V52" s="12"/>
     </row>
     <row r="53" spans="1:23" x14ac:dyDescent="0.25">
       <c r="D53" t="s">
@@ -2976,50 +3009,90 @@
         <v>16</v>
       </c>
       <c r="C61" s="5"/>
-      <c r="D61" s="5"/>
+      <c r="D61" s="5" t="s">
+        <v>14</v>
+      </c>
       <c r="E61" s="5"/>
-      <c r="F61" s="5"/>
+      <c r="F61" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="G61" s="5"/>
-      <c r="H61" s="5"/>
+      <c r="H61" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="I61" s="5"/>
-      <c r="J61" s="5"/>
+      <c r="J61" s="5" t="s">
+        <v>14</v>
+      </c>
       <c r="K61" s="5"/>
-      <c r="L61" s="5"/>
+      <c r="L61" s="5" t="s">
+        <v>14</v>
+      </c>
       <c r="M61" s="5"/>
-      <c r="N61" s="5"/>
+      <c r="N61" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="O61" s="5"/>
-      <c r="P61" s="5"/>
+      <c r="P61" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="Q61" s="5"/>
-      <c r="R61" s="5"/>
+      <c r="R61" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="S61" s="5"/>
-      <c r="T61" s="5"/>
+      <c r="T61" s="5" t="s">
+        <v>14</v>
+      </c>
       <c r="U61" s="5"/>
-      <c r="V61" s="6"/>
+      <c r="V61" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="62" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B62" s="4" t="s">
         <v>17</v>
       </c>
       <c r="C62" s="5"/>
-      <c r="D62" s="5"/>
+      <c r="D62" s="5">
+        <v>-105</v>
+      </c>
       <c r="E62" s="5"/>
-      <c r="F62" s="5"/>
+      <c r="F62" s="5">
+        <v>-225</v>
+      </c>
       <c r="G62" s="5"/>
-      <c r="H62" s="5"/>
+      <c r="H62" s="5">
+        <v>-270</v>
+      </c>
       <c r="I62" s="5"/>
-      <c r="J62" s="5"/>
+      <c r="J62" s="5">
+        <v>-180</v>
+      </c>
       <c r="K62" s="5"/>
-      <c r="L62" s="5"/>
+      <c r="L62" s="5">
+        <v>-170</v>
+      </c>
       <c r="M62" s="5"/>
-      <c r="N62" s="5"/>
+      <c r="N62" s="5">
+        <v>-255</v>
+      </c>
       <c r="O62" s="5"/>
-      <c r="P62" s="5"/>
+      <c r="P62" s="5">
+        <v>-235</v>
+      </c>
       <c r="Q62" s="5"/>
-      <c r="R62" s="5"/>
+      <c r="R62" s="5">
+        <v>-270</v>
+      </c>
       <c r="S62" s="5"/>
-      <c r="T62" s="5"/>
+      <c r="T62" s="5">
+        <v>-475</v>
+      </c>
       <c r="U62" s="5"/>
-      <c r="V62" s="6"/>
+      <c r="V62" s="6">
+        <v>-310</v>
+      </c>
     </row>
     <row r="64" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B64" s="4" t="s">
@@ -3070,83 +3143,83 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="65" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B65" s="4" t="s">
         <v>19</v>
       </c>
       <c r="C65" s="5"/>
-      <c r="D65" s="5" t="e">
+      <c r="D65" s="5">
         <f>IF(D62&gt;0,ROUND(ABS(D64)*(D62/100),2),ROUND(D64/(D62/100),2))</f>
-        <v>#DIV/0!</v>
+        <v>0.95</v>
       </c>
       <c r="E65" s="5"/>
-      <c r="F65" s="5" t="e">
+      <c r="F65" s="5">
         <f>IF(F62&gt;0,ROUND(ABS(F64)*(F62/100),2),ROUND(F64/(F62/100),2))</f>
-        <v>#DIV/0!</v>
+        <v>0.44</v>
       </c>
       <c r="G65" s="5"/>
-      <c r="H65" s="5" t="e">
+      <c r="H65" s="5">
         <f>IF(H62&gt;0,ROUND(ABS(H64)*(H62/100),2),ROUND(H64/(H62/100),2))</f>
-        <v>#DIV/0!</v>
+        <v>0.37</v>
       </c>
       <c r="I65" s="5"/>
-      <c r="J65" s="5" t="e">
+      <c r="J65" s="5">
         <f>IF(J62&gt;0,ROUND(ABS(J64)*(J62/100),2),ROUND(J64/(J62/100),2))</f>
-        <v>#DIV/0!</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="K65" s="5"/>
-      <c r="L65" s="5" t="e">
+      <c r="L65" s="5">
         <f>IF(L62&gt;0,ROUND(ABS(L64)*(L62/100),2),ROUND(L64/(L62/100),2))</f>
-        <v>#DIV/0!</v>
+        <v>0.59</v>
       </c>
       <c r="M65" s="5"/>
-      <c r="N65" s="5" t="e">
+      <c r="N65" s="5">
         <f>IF(N62&gt;0,ROUND(ABS(N64)*(N62/100),2),ROUND(N64/(N62/100),2))</f>
-        <v>#DIV/0!</v>
+        <v>0.39</v>
       </c>
       <c r="O65" s="5"/>
-      <c r="P65" s="5" t="e">
+      <c r="P65" s="5">
         <f>IF(P62&gt;0,ROUND(ABS(P64)*(P62/100),2),ROUND(P64/(P62/100),2))</f>
-        <v>#DIV/0!</v>
+        <v>0.43</v>
       </c>
       <c r="Q65" s="5"/>
-      <c r="R65" s="5" t="e">
+      <c r="R65" s="5">
         <f>IF(R62&gt;0,ROUND(ABS(R64)*(R62/100),2),ROUND(R64/(R62/100),2))</f>
-        <v>#DIV/0!</v>
+        <v>0.37</v>
       </c>
       <c r="S65" s="5"/>
-      <c r="T65" s="5" t="e">
+      <c r="T65" s="5">
         <f>IF(T62&gt;0,ROUND(ABS(T64)*(T62/100),2),ROUND(T64/(T62/100),2))</f>
-        <v>#DIV/0!</v>
+        <v>0.21</v>
       </c>
       <c r="U65" s="5"/>
-      <c r="V65" s="5" t="e">
+      <c r="V65" s="5">
         <f>IF(V62&gt;0,ROUND(ABS(V64)*(V62/100),2),ROUND(V64/(V62/100),2))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W65" s="8" t="e">
+        <v>0.32</v>
+      </c>
+      <c r="W65" s="8">
         <f>SUM(D65:V65)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="66" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4.63</v>
+      </c>
+    </row>
+    <row r="66" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B66" s="4" t="s">
         <v>20</v>
       </c>
       <c r="C66" s="5"/>
       <c r="D66" s="5">
         <f>IF(D61=D59,-D64+D65,0)</f>
-        <v>0</v>
+        <v>1.95</v>
       </c>
       <c r="E66" s="5"/>
       <c r="F66" s="5">
         <f>IF(F61=F59,-F64+F65,0)</f>
-        <v>0</v>
+        <v>1.44</v>
       </c>
       <c r="G66" s="5"/>
       <c r="H66" s="5">
         <f>IF(H61=H59,-H64+H65,0)</f>
-        <v>0</v>
+        <v>1.37</v>
       </c>
       <c r="I66" s="5"/>
       <c r="J66" s="5">
@@ -3161,17 +3234,17 @@
       <c r="M66" s="5"/>
       <c r="N66" s="5">
         <f>IF(N61=N59,-N64+N65,0)</f>
-        <v>0</v>
+        <v>1.3900000000000001</v>
       </c>
       <c r="O66" s="5"/>
       <c r="P66" s="5">
         <f>IF(P61=P59,-P64+P65,0)</f>
-        <v>0</v>
+        <v>1.43</v>
       </c>
       <c r="Q66" s="5"/>
       <c r="R66" s="5">
         <f>IF(R61=R59,-R64+R65,0)</f>
-        <v>0</v>
+        <v>1.37</v>
       </c>
       <c r="S66" s="5"/>
       <c r="T66" s="5">
@@ -3181,31 +3254,423 @@
       <c r="U66" s="5"/>
       <c r="V66" s="6">
         <f>IF(V61=V59,-V64+V65,0)</f>
-        <v>0</v>
+        <v>1.32</v>
       </c>
       <c r="W66" s="9">
         <f>SUM(D66:V66)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="2:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>10.27</v>
+      </c>
+    </row>
+    <row r="67" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="W67" s="7">
         <f>W64+W66</f>
+        <v>0.26999999999999957</v>
+      </c>
+    </row>
+    <row r="68" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="U68" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="V68" s="13"/>
+      <c r="W68" s="11">
+        <f>W51+W67</f>
+        <v>1.0899999999999999</v>
+      </c>
+    </row>
+    <row r="69" spans="1:23" ht="24" x14ac:dyDescent="0.4">
+      <c r="D69" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E69" s="12"/>
+      <c r="F69" s="12"/>
+      <c r="G69" s="12"/>
+      <c r="H69" s="12"/>
+      <c r="I69" s="12"/>
+      <c r="J69" s="12"/>
+      <c r="K69" s="12"/>
+      <c r="L69" s="12"/>
+      <c r="M69" s="12"/>
+      <c r="N69" s="12"/>
+      <c r="O69" s="12"/>
+      <c r="P69" s="12"/>
+      <c r="Q69" s="12"/>
+      <c r="R69" s="12"/>
+      <c r="S69" s="12"/>
+      <c r="T69" s="12"/>
+      <c r="U69" s="12"/>
+      <c r="V69" s="12"/>
+    </row>
+    <row r="70" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="D70" t="s">
+        <v>58</v>
+      </c>
+      <c r="F70" t="s">
+        <v>59</v>
+      </c>
+      <c r="H70" t="s">
+        <v>60</v>
+      </c>
+      <c r="J70" t="s">
+        <v>61</v>
+      </c>
+      <c r="L70" t="s">
+        <v>62</v>
+      </c>
+      <c r="N70" t="s">
+        <v>63</v>
+      </c>
+      <c r="P70" t="s">
+        <v>64</v>
+      </c>
+      <c r="R70" t="s">
+        <v>65</v>
+      </c>
+      <c r="T70" t="s">
+        <v>66</v>
+      </c>
+      <c r="V70" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="71" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>3.5</v>
+      </c>
+      <c r="B71" s="1">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="72" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>2.5</v>
+      </c>
+      <c r="B72" s="1">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="73" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>3.5</v>
+      </c>
+      <c r="B73" s="1">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="74" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>2.5</v>
+      </c>
+      <c r="B74" s="1">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="76" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B76" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C76" s="5"/>
+      <c r="D76" s="5"/>
+      <c r="E76" s="5"/>
+      <c r="F76" s="5"/>
+      <c r="G76" s="5"/>
+      <c r="H76" s="5"/>
+      <c r="I76" s="5"/>
+      <c r="J76" s="5"/>
+      <c r="K76" s="5"/>
+      <c r="L76" s="5"/>
+      <c r="M76" s="5"/>
+      <c r="N76" s="5"/>
+      <c r="O76" s="5"/>
+      <c r="P76" s="5"/>
+      <c r="Q76" s="5"/>
+      <c r="R76" s="5"/>
+      <c r="S76" s="5"/>
+      <c r="T76" s="5"/>
+      <c r="U76" s="5"/>
+      <c r="V76" s="6"/>
+    </row>
+    <row r="77" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B77" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C77" s="5"/>
+      <c r="D77" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="E77" s="5"/>
+      <c r="F77" s="5">
+        <v>3.5</v>
+      </c>
+      <c r="G77" s="5"/>
+      <c r="H77" s="5">
+        <v>3.5</v>
+      </c>
+      <c r="I77" s="5"/>
+      <c r="J77" s="5">
+        <v>3.5</v>
+      </c>
+      <c r="K77" s="5"/>
+      <c r="L77" s="5">
+        <v>3.5</v>
+      </c>
+      <c r="M77" s="5"/>
+      <c r="N77" s="5">
+        <v>3.5</v>
+      </c>
+      <c r="O77" s="5"/>
+      <c r="P77" s="5">
+        <v>3.5</v>
+      </c>
+      <c r="Q77" s="5"/>
+      <c r="R77" s="5">
+        <v>3.5</v>
+      </c>
+      <c r="S77" s="5"/>
+      <c r="T77" s="5">
+        <v>3.5</v>
+      </c>
+      <c r="U77" s="5"/>
+      <c r="V77" s="6">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B78" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C78" s="5"/>
+      <c r="D78" s="5"/>
+      <c r="E78" s="5"/>
+      <c r="F78" s="5"/>
+      <c r="G78" s="5"/>
+      <c r="H78" s="5"/>
+      <c r="I78" s="5"/>
+      <c r="J78" s="5"/>
+      <c r="K78" s="5"/>
+      <c r="L78" s="5"/>
+      <c r="M78" s="5"/>
+      <c r="N78" s="5"/>
+      <c r="O78" s="5"/>
+      <c r="P78" s="5"/>
+      <c r="Q78" s="5"/>
+      <c r="R78" s="5"/>
+      <c r="S78" s="5"/>
+      <c r="T78" s="5"/>
+      <c r="U78" s="5"/>
+      <c r="V78" s="6"/>
+    </row>
+    <row r="79" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B79" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C79" s="5"/>
+      <c r="D79" s="5"/>
+      <c r="E79" s="5"/>
+      <c r="F79" s="5"/>
+      <c r="G79" s="5"/>
+      <c r="H79" s="5"/>
+      <c r="I79" s="5"/>
+      <c r="J79" s="5"/>
+      <c r="K79" s="5"/>
+      <c r="L79" s="5"/>
+      <c r="M79" s="5"/>
+      <c r="N79" s="5"/>
+      <c r="O79" s="5"/>
+      <c r="P79" s="5"/>
+      <c r="Q79" s="5"/>
+      <c r="R79" s="5"/>
+      <c r="S79" s="5"/>
+      <c r="T79" s="5"/>
+      <c r="U79" s="5"/>
+      <c r="V79" s="6"/>
+    </row>
+    <row r="81" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B81" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C81" s="5"/>
+      <c r="D81" s="5">
+        <v>-1</v>
+      </c>
+      <c r="E81" s="5"/>
+      <c r="F81" s="5">
+        <v>-1</v>
+      </c>
+      <c r="G81" s="5"/>
+      <c r="H81" s="5">
+        <v>-1</v>
+      </c>
+      <c r="I81" s="5"/>
+      <c r="J81" s="5">
+        <v>-1</v>
+      </c>
+      <c r="K81" s="5"/>
+      <c r="L81" s="5">
+        <v>-1</v>
+      </c>
+      <c r="M81" s="5"/>
+      <c r="N81" s="5">
+        <v>-1</v>
+      </c>
+      <c r="O81" s="5"/>
+      <c r="P81" s="5">
+        <v>-1</v>
+      </c>
+      <c r="Q81" s="5"/>
+      <c r="R81" s="5">
+        <v>-1</v>
+      </c>
+      <c r="S81" s="5"/>
+      <c r="T81" s="5">
+        <v>-1</v>
+      </c>
+      <c r="U81" s="5"/>
+      <c r="V81" s="6">
+        <v>-1</v>
+      </c>
+      <c r="W81" s="8">
+        <f>SUM(D81:V81)</f>
         <v>-10</v>
       </c>
     </row>
-    <row r="68" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="U68" s="12" t="s">
+    <row r="82" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B82" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C82" s="5"/>
+      <c r="D82" s="5" t="e">
+        <f>IF(D79&gt;0,ROUND(ABS(D81)*(D79/100),2),ROUND(D81/(D79/100),2))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E82" s="5"/>
+      <c r="F82" s="5" t="e">
+        <f>IF(F79&gt;0,ROUND(ABS(F81)*(F79/100),2),ROUND(F81/(F79/100),2))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G82" s="5"/>
+      <c r="H82" s="5" t="e">
+        <f>IF(H79&gt;0,ROUND(ABS(H81)*(H79/100),2),ROUND(H81/(H79/100),2))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I82" s="5"/>
+      <c r="J82" s="5" t="e">
+        <f>IF(J79&gt;0,ROUND(ABS(J81)*(J79/100),2),ROUND(J81/(J79/100),2))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="K82" s="5"/>
+      <c r="L82" s="5" t="e">
+        <f>IF(L79&gt;0,ROUND(ABS(L81)*(L79/100),2),ROUND(L81/(L79/100),2))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="M82" s="5"/>
+      <c r="N82" s="5" t="e">
+        <f>IF(N79&gt;0,ROUND(ABS(N81)*(N79/100),2),ROUND(N81/(N79/100),2))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="O82" s="5"/>
+      <c r="P82" s="5" t="e">
+        <f>IF(P79&gt;0,ROUND(ABS(P81)*(P79/100),2),ROUND(P81/(P79/100),2))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Q82" s="5"/>
+      <c r="R82" s="5" t="e">
+        <f>IF(R79&gt;0,ROUND(ABS(R81)*(R79/100),2),ROUND(R81/(R79/100),2))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="S82" s="5"/>
+      <c r="T82" s="5" t="e">
+        <f>IF(T79&gt;0,ROUND(ABS(T81)*(T79/100),2),ROUND(T81/(T79/100),2))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U82" s="5"/>
+      <c r="V82" s="5" t="e">
+        <f>IF(V79&gt;0,ROUND(ABS(V81)*(V79/100),2),ROUND(V81/(V79/100),2))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W82" s="8" t="e">
+        <f>SUM(D82:V82)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="83" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B83" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C83" s="5"/>
+      <c r="D83" s="5" t="e">
+        <f>IF(D78=D76,-D81+D82,0)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E83" s="5"/>
+      <c r="F83" s="5" t="e">
+        <f>IF(F78=F76,-F81+F82,0)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G83" s="5"/>
+      <c r="H83" s="5" t="e">
+        <f>IF(H78=H76,-H81+H82,0)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I83" s="5"/>
+      <c r="J83" s="5" t="e">
+        <f>IF(J78=J76,-J81+J82,0)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="K83" s="5"/>
+      <c r="L83" s="5" t="e">
+        <f>IF(L78=L76,-L81+L82,0)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="M83" s="5"/>
+      <c r="N83" s="5" t="e">
+        <f>IF(N78=N76,-N81+N82,0)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="O83" s="5"/>
+      <c r="P83" s="5" t="e">
+        <f>IF(P78=P76,-P81+P82,0)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Q83" s="5"/>
+      <c r="R83" s="5" t="e">
+        <f>IF(R78=R76,-R81+R82,0)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="S83" s="5"/>
+      <c r="T83" s="5" t="e">
+        <f>IF(T78=T76,-T81+T82,0)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U83" s="5"/>
+      <c r="V83" s="6" t="e">
+        <f>IF(V78=V76,-V81+V82,0)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W83" s="9" t="e">
+        <f>SUM(D83:V83)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="84" spans="2:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="W84" s="7" t="e">
+        <f>W81+W83</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="85" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="U85" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="V68" s="12"/>
-      <c r="W68" s="11" t="e">
-        <f>#REF!+W67</f>
-        <v>#REF!</v>
+      <c r="V85" s="13"/>
+      <c r="W85" s="11" t="e">
+        <f>W68+W84</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="10">
+    <mergeCell ref="D69:V69"/>
+    <mergeCell ref="U85:V85"/>
     <mergeCell ref="D52:V52"/>
     <mergeCell ref="U68:V68"/>
     <mergeCell ref="U51:V51"/>

</xml_diff>